<commit_message>
chore(scripts): import EmploiDuTemps sheet + login/parent helpers
- makeImportTemplate: add 5th "EmploiDuTemps" sheet (teacherEmail, day,
  startTime, endTime, durationMin, classe, seance, room, subject)
- importFromTemplate: parse + validate EDT rows (day/time aliases, duration
  fallback), write schedules/{uid}, then rebuild emploiDuTemps aggregate
- syncEmploiDuTemps: carry seance through to emploiDuTemps docs
- add listLogins.js (read-only last-activity report) and quickParent.js
  (create/reset a test parent account)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mojammaa_import_template.xlsx
+++ b/mojammaa_import_template.xlsx
@@ -7,6 +7,7 @@
     <sheet name="Enseignants" sheetId="2" r:id="rId2"/>
     <sheet name="Eleves" sheetId="3" r:id="rId3"/>
     <sheet name="Parents" sheetId="4" r:id="rId4"/>
+    <sheet name="EmploiDuTemps" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -400,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A36"/>
   <cols>
     <col min="1" max="1" width="70.83203125" customWidth="1"/>
   </cols>
@@ -447,117 +448,147 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v/>
+        <v xml:space="preserve">  4) EmploiDuTemps — après Enseignants (teacherEmail doit exister)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>RÈGLES GÉNÉRALES :</v>
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v xml:space="preserve">  • Ne change PAS la ligne d’en-tête (ligne 1 de chaque feuille).</v>
+        <v>RÈGLES GÉNÉRALES :</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v xml:space="preserve">  • Supprime les lignes "EXEMPLE" avant de me renvoyer le fichier.</v>
+        <v xml:space="preserve">  • Ne change PAS la ligne d’en-tête (ligne 1 de chaque feuille).</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v xml:space="preserve">  • Une ligne = une personne.</v>
+        <v xml:space="preserve">  • Supprime les lignes "EXEMPLE" avant de me renvoyer le fichier.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v xml:space="preserve">  • Colonnes "classes"/"enfants" multiples : séparer par une virgule.</v>
+        <v xml:space="preserve">  • Une ligne = une personne.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v xml:space="preserve">  • Dates au format AAAA-MM-JJ (ex : 2011-09-15).</v>
+        <v xml:space="preserve">  • Colonnes "classes"/"enfants" multiples : séparer par une virgule.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v xml:space="preserve">  • password : laisser VIDE = mot de passe par défaut "&lt;email&gt;1234".</v>
+        <v xml:space="preserve">  • Dates au format AAAA-MM-JJ (ex : 2011-09-15).</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v/>
+        <v xml:space="preserve">  • password : laisser VIDE = mot de passe par défaut "&lt;email&gt;1234".</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>FEUILLE "Enseignants" :</v>
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v xml:space="preserve">  email, password(optionnel), nom, prenom, matiere,</v>
+        <v>FEUILLE "Enseignants" :</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v xml:space="preserve">  cycle (primaire | college), classes (ex: 3APIC-1,3APIC-2)</v>
+        <v xml:space="preserve">  email, password(optionnel), nom, prenom, matiere,</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v/>
+        <v xml:space="preserve">  cycle (primaire | college), classes (ex: 3APIC-1,3APIC-2)</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>FEUILLE "Eleves" :</v>
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v xml:space="preserve">  codeMassar (identifiant unique, ex: A171010188), nom (arabe),</v>
+        <v>FEUILLE "Eleves" :</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v xml:space="preserve">  prenom (arabe), nomLatin, prenomLatin, classe (ex: 3APIC-1),</v>
+        <v xml:space="preserve">  codeMassar (identifiant unique, ex: A171010188), nom (arabe),</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v xml:space="preserve">  niveau (ex: 3APIC), dateNaissance (AAAA-MM-JJ)</v>
+        <v xml:space="preserve">  prenom (arabe), nomLatin, prenomLatin, classe (ex: 3APIC-1),</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v xml:space="preserve">  → nomComplet est généré automatiquement (nom + prenom).</v>
+        <v xml:space="preserve">  niveau (ex: 3APIC), dateNaissance (AAAA-MM-JJ)</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v/>
+        <v xml:space="preserve">  → nomComplet est généré automatiquement (nom + prenom).</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>FEUILLE "Parents" :</v>
+        <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v xml:space="preserve">  email, password(optionnel), nom, prenom,</v>
+        <v>FEUILLE "Parents" :</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
+        <v xml:space="preserve">  email, password(optionnel), nom, prenom,</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
         <v xml:space="preserve">  enfants_codeMassar (codes MASSAR des enfants, séparés par virgule)</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>FEUILLE "EmploiDuTemps" :</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v xml:space="preserve">  teacherEmail, day (monday..saturday ou lundi..samedi), startTime, endTime,</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v xml:space="preserve">  durationMin, classe, seance (S1..S6), room, subject</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v xml:space="preserve">  → Une ligne = un créneau hebdomadaire.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A36"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -751,4 +782,84 @@
     <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I2"/>
+  <cols>
+    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>teacherEmail</v>
+      </c>
+      <c r="B1" t="str">
+        <v>day</v>
+      </c>
+      <c r="C1" t="str">
+        <v>startTime</v>
+      </c>
+      <c r="D1" t="str">
+        <v>endTime</v>
+      </c>
+      <c r="E1" t="str">
+        <v>durationMin</v>
+      </c>
+      <c r="F1" t="str">
+        <v>classe</v>
+      </c>
+      <c r="G1" t="str">
+        <v>seance</v>
+      </c>
+      <c r="H1" t="str">
+        <v>room</v>
+      </c>
+      <c r="I1" t="str">
+        <v>subject</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>EXEMPLE prof@gmail.com</v>
+      </c>
+      <c r="B2" t="str">
+        <v>monday</v>
+      </c>
+      <c r="C2" t="str">
+        <v>08:30</v>
+      </c>
+      <c r="D2" t="str">
+        <v>09:30</v>
+      </c>
+      <c r="E2">
+        <v>60</v>
+      </c>
+      <c r="F2" t="str">
+        <v>3APIC-1</v>
+      </c>
+      <c r="G2" t="str">
+        <v>S1</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Salle 4</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Mathématiques</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>